<commit_message>
Added Secondary Owner to database schema
</commit_message>
<xml_diff>
--- a/Jackson Court Resident Directory.xlsx
+++ b/Jackson Court Resident Directory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10222"/>
   <workbookPr showInkAnnotation="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/19b0eb284687b6b8/Alpine Tournament Committee/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/19b0eb284687b6b8/Jackson Court Condo HOA/HOA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:40000001_{68840BA9-4FD9-D846-B0BF-FC0E31165DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0491CC1-67F9-284B-9749-A3768C4A36D1}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:40000001_{68840BA9-4FD9-D846-B0BF-FC0E31165DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C10C9955-6B8F-A046-968A-2D3EA7ACC750}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="17200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,24 +24,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Email Address</t>
-  </si>
-  <si>
-    <t>Owner(s) Name</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="64">
   <si>
     <t>Unit</t>
   </si>
   <si>
-    <t>David Ruggieri
-Twenty Eight Court Street, LLC</t>
-  </si>
-  <si>
     <t>401-440-3984</t>
   </si>
   <si>
@@ -123,22 +110,10 @@
     <t>aymanyounan61@gmail.com</t>
   </si>
   <si>
-    <t>Ayman Youan
-Marian Younan</t>
-  </si>
-  <si>
     <t>Fotini Papadopoulou</t>
   </si>
   <si>
     <t>fpapadop@bidmc.harvard.edu</t>
-  </si>
-  <si>
-    <t>Davide Mancone
-Heather Nary</t>
-  </si>
-  <si>
-    <t>774-581-1737
-774-581-6558</t>
   </si>
   <si>
     <t>wmcdermott99@gmail.com</t>
@@ -169,22 +144,10 @@
 amandarjoyce108@gmail.com</t>
   </si>
   <si>
-    <t>mancone79@gmail.com
-hmancone79@gmail.com</t>
-  </si>
-  <si>
     <t>Don Brown
 Melissa Brown</t>
   </si>
   <si>
-    <t>Erik Freitas
-Alyssa Burke</t>
-  </si>
-  <si>
-    <t>erikfreitasmedia@gmail.com
-alyssamarie363@gmail.com</t>
-  </si>
-  <si>
     <t>Chris</t>
   </si>
   <si>
@@ -196,6 +159,69 @@
   </si>
   <si>
     <t>508-642-1830</t>
+  </si>
+  <si>
+    <t>Owner 1 Name</t>
+  </si>
+  <si>
+    <t>Owner 1 Phone</t>
+  </si>
+  <si>
+    <t>Owner 1 Email Address</t>
+  </si>
+  <si>
+    <t>Owner 2 Name</t>
+  </si>
+  <si>
+    <t>Owner 2 Phone</t>
+  </si>
+  <si>
+    <t>Owner 2 Email Address</t>
+  </si>
+  <si>
+    <t>Alyssa Burke</t>
+  </si>
+  <si>
+    <t>alyssamarie363@gmail.com</t>
+  </si>
+  <si>
+    <t>erikfreitasmedia@gmail.com</t>
+  </si>
+  <si>
+    <t>Heather Mancone</t>
+  </si>
+  <si>
+    <t>508-208-4302</t>
+  </si>
+  <si>
+    <t>hmancone79@gmail.com</t>
+  </si>
+  <si>
+    <t>mancone79@gmail.com</t>
+  </si>
+  <si>
+    <t>Davide Mancone</t>
+  </si>
+  <si>
+    <t>Brett Argall</t>
+  </si>
+  <si>
+    <t>David Ruggieri</t>
+  </si>
+  <si>
+    <t>Marian Younan</t>
+  </si>
+  <si>
+    <t>Ayman Youan</t>
+  </si>
+  <si>
+    <t>774-581-6558</t>
+  </si>
+  <si>
+    <t>774-581-1737</t>
+  </si>
+  <si>
+    <t>Erik Freitas</t>
   </si>
 </sst>
 </file>
@@ -370,6 +396,15 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -378,15 +413,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -398,7 +424,19 @@
     <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Zip Code" xfId="3" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="15">
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -422,15 +460,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -453,6 +482,12 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -503,10 +538,10 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="Membership List" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Membership List" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="11"/>
-      <tableStyleElement type="headerRow" dxfId="10"/>
-      <tableStyleElement type="firstRowStripe" dxfId="9"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="8"/>
+      <tableStyleElement type="wholeTable" dxfId="14"/>
+      <tableStyleElement type="headerRow" dxfId="13"/>
+      <tableStyleElement type="firstRowStripe" dxfId="12"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="11"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -589,14 +624,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="List" displayName="List" ref="A2:H13" totalsRowShown="0" headerRowCellStyle="Normal">
-  <autoFilter ref="A2:H13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Unit" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{CE5AE129-FADC-DB46-93EA-DABEFA0AA4C1}" name="Owner(s) Name" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Phone" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Email Address" dataDxfId="0"/>
-    <tableColumn id="16" xr3:uid="{0EE0B542-D508-E84E-A884-54700D6F4261}" name="Renter (if applicable)" dataDxfId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="List" displayName="List" ref="A2:K13" totalsRowShown="0" headerRowCellStyle="Normal">
+  <autoFilter ref="A2:K13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Unit" dataDxfId="10"/>
+    <tableColumn id="14" xr3:uid="{CE5AE129-FADC-DB46-93EA-DABEFA0AA4C1}" name="Owner 1 Name" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Owner 1 Phone" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Owner 1 Email Address" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{810F8596-78CE-9D41-B835-8EB0287C4BAA}" name="Owner 2 Name" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{93BE44DE-9D86-4E47-8B56-86BA0C34F135}" name="Owner 2 Phone" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{96F45AB7-DEEF-1149-AFFE-1CC983455010}" name="Owner 2 Email Address" dataDxfId="2"/>
+    <tableColumn id="16" xr3:uid="{0EE0B542-D508-E84E-A884-54700D6F4261}" name="Renter (if applicable)" dataDxfId="6"/>
     <tableColumn id="15" xr3:uid="{519DC660-07F9-D846-BDAA-78BBE651A4C1}" name="Renter Name" dataDxfId="5"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Phone2" dataDxfId="4"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Email" dataDxfId="3"/>
@@ -901,294 +939,355 @@
     <tabColor theme="4" tint="0.39997558519241921"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="29.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="29.1640625" customWidth="1"/>
-    <col min="5" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="32.6640625" customWidth="1"/>
+    <col min="4" max="7" width="29.1640625" customWidth="1"/>
+    <col min="8" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="11" max="11" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="56.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="13"/>
+    <row r="1" spans="1:11" ht="56.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="16"/>
     </row>
-    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" t="s">
-        <v>10</v>
+      <c r="I2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H3" s="5"/>
+      <c r="J3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" s="5"/>
     </row>
-    <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="8"/>
+        <v>20</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
       <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="7"/>
     </row>
-    <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2">
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>41</v>
+      <c r="D5" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3">
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="8"/>
+        <v>62</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="12"/>
       <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="7"/>
     </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="3">
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>44</v>
+        <v>1</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3">
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="8"/>
+        <v>15</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
       <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="7"/>
     </row>
-    <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="3">
         <v>7</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
       <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="3">
         <v>8</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="8"/>
+        <v>40</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>54</v>
+      </c>
       <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="7"/>
     </row>
-    <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3">
         <v>9</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="8"/>
+        <v>41</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
       <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3">
         <v>10</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
+        <v>17</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
       <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="7"/>
     </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>11</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="H13" s="9"/>
+        <v>18</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="K13" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="6">
+  <dataValidations count="6">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Create a Membership List in this worksheet. Title of this worksheet is in this cell. Enter Club Name within brackets in this cell" sqref="A1" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Member Name in this column under this heading. Use heading filters to find specific entries" sqref="A2:B2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Phone number in this column under this heading" sqref="C2" xr:uid="{00000000-0002-0000-0000-000005000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Email Address in this column under this heading" sqref="D2:F2" xr:uid="{00000000-0002-0000-0000-00000A000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Fax number in this column under this heading" sqref="G2" xr:uid="{00000000-0002-0000-0000-00000B000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Notes in this column under this heading" sqref="H2" xr:uid="{00000000-0002-0000-0000-00000C000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Email Address in this column under this heading" sqref="D2:I2" xr:uid="{00000000-0002-0000-0000-00000A000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Fax number in this column under this heading" sqref="J2" xr:uid="{00000000-0002-0000-0000-00000B000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Notes in this column under this heading" sqref="K2" xr:uid="{00000000-0002-0000-0000-00000C000000}"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>